<commit_message>
Mise à jour du dernier package terminologies (#132) 58438319289c40499962ea7353ce40a139082ac3
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-mesures-bundle-flux-alimentation.xlsx
+++ b/main/ig/StructureDefinition-mesures-bundle-flux-alimentation.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-07-21T12:31:31+00:00</t>
+    <t>2025-10-13T07:29:09+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -361,7 +361,7 @@
     <t>A human language.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/languages</t>
+    <t>http://hl7.org/fhir/ValueSet/languages|4.0.1</t>
   </si>
   <si>
     <t>Resource.language</t>

</xml_diff>